<commit_message>
New Skill Platform, Loaded Effects
</commit_message>
<xml_diff>
--- a/Src/Assets/StreamingAssets/Common/Tables/Tables/ActionDefine.xlsx
+++ b/Src/Assets/StreamingAssets/Common/Tables/Tables/ActionDefine.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CCA\Src\Assets\StreamingAssets\Common\Tables\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A9B18D-F055-4849-B520-F9BA192AFE65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE507FDF-E80A-4D55-9CFA-AADA6A89E322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="599" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="599" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supply" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="185">
   <si>
     <t>ID</t>
   </si>
@@ -876,6 +876,12 @@
   </si>
   <si>
     <t>Self</t>
+  </si>
+  <si>
+    <t>Possibility</t>
+  </si>
+  <si>
+    <t>[0,0,20]</t>
   </si>
 </sst>
 </file>
@@ -4520,24 +4526,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27ECECD7-19E1-4627-A931-18B44035B88A}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="26.54296875" style="1" customWidth="1"/>
     <col min="2" max="2" width="26.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="15.81640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="96.81640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="96.81640625" style="1" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="18.1796875" style="1" customWidth="1"/>
     <col min="6" max="6" width="19.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" style="1" customWidth="1"/>
     <col min="8" max="8" width="8.90625" style="1"/>
     <col min="9" max="9" width="9.54296875" style="1" customWidth="1"/>
     <col min="10" max="12" width="8.90625" style="1"/>
     <col min="13" max="13" width="15.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.90625" style="1"/>
+    <col min="14" max="14" width="14.453125" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.90625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="2" customFormat="1" ht="14.5" thickTop="1">
+    <row r="1" spans="1:14" s="2" customFormat="1" ht="14.5" thickTop="1">
       <c r="A1" s="31" t="s">
         <v>31</v>
       </c>
@@ -4577,8 +4584,11 @@
       <c r="M1" s="35" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
+      <c r="N1" s="35" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" s="36" t="s">
         <v>52</v>
       </c>
@@ -4618,8 +4628,11 @@
       <c r="M2" s="37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:13">
+      <c r="N2" s="37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" s="36" t="s">
         <v>54</v>
       </c>
@@ -4659,8 +4672,11 @@
       <c r="M3" s="37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:13">
+      <c r="N3" s="37">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" s="36" t="s">
         <v>53</v>
       </c>
@@ -4700,8 +4716,11 @@
       <c r="M4" s="37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:13">
+      <c r="N4" s="37">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" s="36" t="s">
         <v>55</v>
       </c>
@@ -4741,8 +4760,11 @@
       <c r="M5" s="37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:13">
+      <c r="N5" s="37">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" s="36" t="s">
         <v>67</v>
       </c>
@@ -4782,8 +4804,11 @@
       <c r="M6" s="37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:13">
+      <c r="N6" s="37">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" s="36" t="s">
         <v>65</v>
       </c>
@@ -4823,8 +4848,11 @@
       <c r="M7" s="37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" s="29" customFormat="1">
+      <c r="N7" s="37">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" s="29" customFormat="1">
       <c r="A8" s="38" t="s">
         <v>96</v>
       </c>
@@ -4838,7 +4866,7 @@
         <v>45</v>
       </c>
       <c r="E8" s="41" t="s">
-        <v>144</v>
+        <v>184</v>
       </c>
       <c r="F8" s="40" t="s">
         <v>29</v>
@@ -4864,8 +4892,11 @@
       <c r="M8" s="42" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:13">
+      <c r="N8" s="42">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" s="36" t="s">
         <v>56</v>
       </c>
@@ -4905,8 +4936,11 @@
       <c r="M9" s="37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:13">
+      <c r="N9" s="37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" s="43" t="s">
         <v>57</v>
       </c>
@@ -4946,8 +4980,11 @@
       <c r="M10" s="47" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:13">
+      <c r="N10" s="47">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" s="36" t="s">
         <v>58</v>
       </c>
@@ -4987,8 +5024,11 @@
       <c r="M11" s="37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:13">
+      <c r="N11" s="37">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" s="43" t="s">
         <v>78</v>
       </c>
@@ -5026,8 +5066,11 @@
       <c r="M12" s="47" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:13">
+      <c r="N12" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
       <c r="A13" s="36" t="s">
         <v>59</v>
       </c>
@@ -5067,8 +5110,11 @@
       <c r="M13" s="37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:13">
+      <c r="N13" s="37">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
       <c r="A14" s="43" t="s">
         <v>60</v>
       </c>
@@ -5108,8 +5154,11 @@
       <c r="M14" s="47" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:13">
+      <c r="N14" s="47">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
       <c r="A15" s="36" t="s">
         <v>61</v>
       </c>
@@ -5149,8 +5198,11 @@
       <c r="M15" s="37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" s="29" customFormat="1">
+      <c r="N15" s="37">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" s="29" customFormat="1">
       <c r="A16" s="38" t="s">
         <v>97</v>
       </c>
@@ -5190,8 +5242,11 @@
       <c r="M16" s="42" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" s="30" customFormat="1" ht="28">
+      <c r="N16" s="42">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" s="30" customFormat="1" ht="28">
       <c r="A17" s="38" t="s">
         <v>137</v>
       </c>
@@ -5231,8 +5286,11 @@
       <c r="M17" s="48" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" s="29" customFormat="1" ht="31.25" customHeight="1" thickBot="1">
+      <c r="N17" s="48">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" s="29" customFormat="1" ht="31.25" customHeight="1" thickBot="1">
       <c r="A18" s="49" t="s">
         <v>131</v>
       </c>
@@ -5272,8 +5330,11 @@
       <c r="M18" s="52" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" ht="14.5" thickTop="1"/>
+      <c r="N18" s="52">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="14.5" thickTop="1"/>
   </sheetData>
   <phoneticPr fontId="13" type="noConversion"/>
   <conditionalFormatting sqref="F2:F18 F19:G59">
@@ -5286,7 +5347,7 @@
       <formula>$F17="Self"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M78">
+  <conditionalFormatting sqref="M2:M78 N2:N18">
     <cfRule type="expression" dxfId="65" priority="1">
       <formula>$M2="False"</formula>
     </cfRule>

</xml_diff>

<commit_message>
RougeMap Automatically Generated, Relic Logic completed
</commit_message>
<xml_diff>
--- a/Src/Assets/StreamingAssets/Common/Tables/Tables/ActionDefine.xlsx
+++ b/Src/Assets/StreamingAssets/Common/Tables/Tables/ActionDefine.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook" updateLinks="always"/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12080" tabRatio="599" activeTab="1"/>
+    <workbookView windowWidth="25600" windowHeight="12080" tabRatio="599"/>
   </bookViews>
   <sheets>
     <sheet name="Supply" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="176">
   <si>
     <t>Key</t>
   </si>
@@ -69,6 +69,9 @@
     <t>isBasic</t>
   </si>
   <si>
+    <t>Tags</t>
+  </si>
+  <si>
     <t>bullet</t>
   </si>
   <si>
@@ -87,6 +90,9 @@
     <t>[0,1,0]</t>
   </si>
   <si>
+    <t>["Bullet"]</t>
+  </si>
+  <si>
     <t>double_bullet</t>
   </si>
   <si>
@@ -111,6 +117,9 @@
     <t>[0,0,1]</t>
   </si>
   <si>
+    <t>["Sword"]</t>
+  </si>
+  <si>
     <t>double_sword</t>
   </si>
   <si>
@@ -165,9 +174,6 @@
     <t>Damage</t>
   </si>
   <si>
-    <t>Tags</t>
-  </si>
-  <si>
     <t>stab</t>
   </si>
   <si>
@@ -180,9 +186,6 @@
     <t>Enemy</t>
   </si>
   <si>
-    <t>[Sword]</t>
-  </si>
-  <si>
     <t>cleave</t>
   </si>
   <si>
@@ -198,7 +201,7 @@
     <t>光剑</t>
   </si>
   <si>
-    <t>[Sword,Light]</t>
+    <t>["Sword","Light"]</t>
   </si>
   <si>
     <t>laser_cleave</t>
@@ -255,9 +258,6 @@
     <t>对应防御：挡</t>
   </si>
   <si>
-    <t>[Bullet]</t>
-  </si>
-  <si>
     <t>double_shoot</t>
   </si>
   <si>
@@ -273,7 +273,7 @@
     <t>激光枪</t>
   </si>
   <si>
-    <t>[Bullet,Light]</t>
+    <t>["Bullet","Light"]</t>
   </si>
   <si>
     <t>laser_cannon</t>
@@ -384,6 +384,9 @@
       </rPr>
       <t>和单发子弹类攻击</t>
     </r>
+  </si>
+  <si>
+    <t>[]</t>
   </si>
   <si>
     <t>double_block</t>
@@ -796,7 +799,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="0_ "/>
   </numFmts>
-  <fonts count="42">
+  <fonts count="40">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1005,11 +1008,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="12"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -1019,13 +1017,6 @@
       <color theme="1"/>
       <name val="微软雅黑"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1062,8 +1053,16 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <u/>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="134"/>
     </font>
@@ -1076,21 +1075,13 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="45">
+  <fills count="41">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1273,12 +1264,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1337,26 +1322,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="26">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -1414,6 +1381,19 @@
       <left style="thick">
         <color auto="1"/>
       </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thick">
         <color auto="1"/>
       </right>
@@ -1514,32 +1494,6 @@
     </border>
     <border>
       <left/>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thick">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="thin">
         <color auto="1"/>
@@ -1553,9 +1507,7 @@
       <left style="thick">
         <color auto="1"/>
       </left>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
+      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -1699,7 +1651,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="18" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="17" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1711,34 +1663,34 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1792,69 +1744,69 @@
     <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="34" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="35" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1883,6 +1835,9 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="57" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1925,12 +1880,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1967,13 +1922,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1982,31 +1937,28 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2021,10 +1973,10 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2039,31 +1991,19 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2072,7 +2012,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="9" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="3" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2087,25 +2027,25 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2467,6 +2407,13 @@
       </border>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <name val="宋体"/>
         <scheme val="none"/>
@@ -2765,13 +2712,6 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="8" tint="-0.249946592608417"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3576,9 +3516,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="表1" displayName="表1" ref="A1:L9" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L9" etc:filterBottomFollowUsedRange="0"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="表1" displayName="表1" ref="A1:M9" totalsRowShown="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:M9" etc:filterBottomFollowUsedRange="0"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Key" dataDxfId="0"/>
     <tableColumn id="3" name="ID" dataDxfId="1"/>
     <tableColumn id="5" name="Name" dataDxfId="2"/>
@@ -3591,28 +3531,29 @@
     <tableColumn id="7" name="Target" dataDxfId="9"/>
     <tableColumn id="8" name="isCopy" dataDxfId="10"/>
     <tableColumn id="9" name="isBasic" dataDxfId="11"/>
+    <tableColumn id="12" name="Tags"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="表1_3" displayName="表1_3" ref="A1:N16" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N16" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="表1_3" displayName="表1_3" ref="A1:N18" totalsRowShown="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N18" etc:filterBottomFollowUsedRange="0"/>
   <tableColumns count="14">
-    <tableColumn id="1" name="Key" dataDxfId="12"/>
-    <tableColumn id="3" name="ID" dataDxfId="13"/>
-    <tableColumn id="5" name="Name" dataDxfId="14"/>
-    <tableColumn id="24" name="Description" dataDxfId="15"/>
-    <tableColumn id="2" name="Costs" dataDxfId="16"/>
-    <tableColumn id="11" name="TargetType" dataDxfId="17"/>
+    <tableColumn id="1" name="Key" dataDxfId="13"/>
+    <tableColumn id="3" name="ID" dataDxfId="14"/>
+    <tableColumn id="5" name="Name" dataDxfId="15"/>
+    <tableColumn id="24" name="Description" dataDxfId="16"/>
+    <tableColumn id="2" name="Costs" dataDxfId="17"/>
+    <tableColumn id="11" name="TargetType" dataDxfId="18"/>
     <tableColumn id="10" name="MaxTarget"/>
-    <tableColumn id="6" name="CD" dataDxfId="18"/>
-    <tableColumn id="27" name="Level" dataDxfId="19"/>
-    <tableColumn id="4" name="Damage" dataDxfId="20"/>
-    <tableColumn id="7" name="Target" dataDxfId="21"/>
-    <tableColumn id="8" name="isCopy" dataDxfId="22"/>
-    <tableColumn id="9" name="isBasic" dataDxfId="23"/>
+    <tableColumn id="6" name="CD" dataDxfId="19"/>
+    <tableColumn id="27" name="Level" dataDxfId="20"/>
+    <tableColumn id="4" name="Damage" dataDxfId="21"/>
+    <tableColumn id="7" name="Target" dataDxfId="22"/>
+    <tableColumn id="8" name="isCopy" dataDxfId="23"/>
+    <tableColumn id="9" name="isBasic" dataDxfId="24"/>
     <tableColumn id="12" name="Tags"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3620,9 +3561,9 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="表1_4" displayName="表1_4" ref="A1:K5" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:K5" etc:filterBottomFollowUsedRange="0"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="表1_4" displayName="表1_4" ref="A1:L5" totalsRowShown="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L5" etc:filterBottomFollowUsedRange="0"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="Key" dataDxfId="27"/>
     <tableColumn id="3" name="ID" dataDxfId="28"/>
     <tableColumn id="5" name="Name" dataDxfId="29"/>
@@ -3634,15 +3575,16 @@
     <tableColumn id="6" name="Target" dataDxfId="35"/>
     <tableColumn id="7" name="isCopy" dataDxfId="36"/>
     <tableColumn id="8" name="isBasic" dataDxfId="37"/>
+    <tableColumn id="10" name="Tags"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="表1_45" displayName="表1_45" ref="A1:K5" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:K5" etc:filterBottomFollowUsedRange="0"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="表1_45" displayName="表1_45" ref="A1:L5" totalsRowShown="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L5" etc:filterBottomFollowUsedRange="0"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="Key" dataDxfId="38"/>
     <tableColumn id="3" name="ID" dataDxfId="39"/>
     <tableColumn id="5" name="Name" dataDxfId="40"/>
@@ -3654,15 +3596,16 @@
     <tableColumn id="6" name="Target" dataDxfId="46"/>
     <tableColumn id="7" name="isCopy" dataDxfId="47"/>
     <tableColumn id="8" name="isBasic" dataDxfId="48"/>
+    <tableColumn id="10" name="Tags"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="表1_6" displayName="表1_6" ref="A1:L15" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L15" etc:filterBottomFollowUsedRange="0"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="表1_6" displayName="表1_6" ref="A1:M15" totalsRowShown="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:M15" etc:filterBottomFollowUsedRange="0"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Key" dataDxfId="49"/>
     <tableColumn id="3" name="ID" dataDxfId="50"/>
     <tableColumn id="5" name="Name" dataDxfId="51"/>
@@ -3675,6 +3618,7 @@
     <tableColumn id="2" name="Target" dataDxfId="58"/>
     <tableColumn id="6" name="isCopy" dataDxfId="59"/>
     <tableColumn id="7" name="isBasic" dataDxfId="60"/>
+    <tableColumn id="8" name="Tags"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3967,368 +3911,397 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultColWidth="16.1818181818182" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="19" style="29" customWidth="1"/>
-    <col min="2" max="2" width="22.0909090909091" style="29" customWidth="1"/>
-    <col min="3" max="3" width="12.9090909090909" style="29" customWidth="1"/>
-    <col min="4" max="5" width="14.3636363636364" style="29" customWidth="1"/>
-    <col min="6" max="6" width="11.8181818181818" style="29" customWidth="1"/>
-    <col min="7" max="7" width="18.5454545454545" style="29" customWidth="1"/>
+    <col min="1" max="1" width="19" style="30" customWidth="1"/>
+    <col min="2" max="2" width="22.0909090909091" style="30" customWidth="1"/>
+    <col min="3" max="3" width="12.9090909090909" style="30" customWidth="1"/>
+    <col min="4" max="5" width="14.3636363636364" style="30" customWidth="1"/>
+    <col min="6" max="6" width="11.8181818181818" style="30" customWidth="1"/>
+    <col min="7" max="7" width="18.5454545454545" style="30" customWidth="1"/>
     <col min="8" max="9" width="16.1818181818182" style="1"/>
-    <col min="10" max="10" width="16.1818181818182" style="29"/>
+    <col min="10" max="10" width="16.1818181818182" style="30"/>
     <col min="11" max="16384" width="16.1818181818182" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.75" spans="1:12">
-      <c r="A1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="44" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="44" t="s">
+    <row r="1" ht="14.75" spans="1:13">
+      <c r="A1" s="44" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="44" t="s">
+      <c r="F1" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="44" t="s">
+      <c r="G1" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="46" t="s">
+      <c r="H1" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="47" t="s">
+      <c r="I1" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="44" t="s">
+      <c r="J1" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="44" t="s">
+      <c r="K1" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="48" t="s">
+      <c r="L1" s="49" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
-      <c r="A2" s="70" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="71" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="34" t="s">
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="B2" s="67" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="D2" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="36" t="s">
+      <c r="E2" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="36">
-        <v>1</v>
-      </c>
-      <c r="H2" s="34">
-        <v>0</v>
-      </c>
-      <c r="I2" s="72" t="s">
+      <c r="F2" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="34">
-        <v>0</v>
-      </c>
-      <c r="K2" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="L2" s="50" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" s="70" t="s">
+      <c r="G2" s="37">
+        <v>1</v>
+      </c>
+      <c r="H2" s="35">
+        <v>0</v>
+      </c>
+      <c r="I2" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="71" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="34" t="s">
+      <c r="J2" s="35">
+        <v>0</v>
+      </c>
+      <c r="K2" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="34" t="s">
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="34" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="36" t="s">
+      <c r="B3" s="67" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="36">
-        <v>1</v>
-      </c>
-      <c r="H3" s="34">
-        <v>0</v>
-      </c>
-      <c r="I3" s="72" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="34">
-        <v>0</v>
-      </c>
-      <c r="K3" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="L3" s="50" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="A4" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="71" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="34" t="s">
+      <c r="F3" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="37">
+        <v>1</v>
+      </c>
+      <c r="H3" s="35">
+        <v>0</v>
+      </c>
+      <c r="I3" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="J3" s="35">
+        <v>0</v>
+      </c>
+      <c r="K3" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="34" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="36" t="s">
+      <c r="B4" s="67" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="36">
-        <v>1</v>
-      </c>
-      <c r="H4" s="34">
-        <v>0</v>
-      </c>
-      <c r="I4" s="72" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" s="34">
-        <v>0</v>
-      </c>
-      <c r="K4" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="L4" s="50" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="70" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="71" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="34" t="s">
+      <c r="F4" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="37">
+        <v>1</v>
+      </c>
+      <c r="H4" s="35">
+        <v>0</v>
+      </c>
+      <c r="I4" s="68" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="J4" s="35">
+        <v>0</v>
+      </c>
+      <c r="K4" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="34" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="36" t="s">
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="66" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="67" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="36">
-        <v>1</v>
-      </c>
-      <c r="H5" s="34">
-        <v>0</v>
-      </c>
-      <c r="I5" s="72" t="s">
-        <v>29</v>
-      </c>
-      <c r="J5" s="34">
-        <v>0</v>
-      </c>
-      <c r="K5" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="L5" s="50" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" s="73" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="74" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="75" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="75" t="s">
+      <c r="F5" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="37">
+        <v>1</v>
+      </c>
+      <c r="H5" s="35">
+        <v>0</v>
+      </c>
+      <c r="I5" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="75" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="76" t="s">
+      <c r="J5" s="35">
+        <v>0</v>
+      </c>
+      <c r="K5" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="69" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="70" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="71" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="71" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="76">
-        <v>1</v>
-      </c>
-      <c r="H6" s="75">
-        <v>0</v>
-      </c>
-      <c r="I6" s="77" t="s">
-        <v>33</v>
-      </c>
-      <c r="J6" s="75">
-        <v>0</v>
-      </c>
-      <c r="K6" s="75" t="b">
-        <v>0</v>
-      </c>
-      <c r="L6" s="78" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="70" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="71" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="34" t="s">
+      <c r="F6" s="72" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="72">
+        <v>1</v>
+      </c>
+      <c r="H6" s="71">
+        <v>0</v>
+      </c>
+      <c r="I6" s="73" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="34" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="36" t="s">
+      <c r="J6" s="71">
+        <v>0</v>
+      </c>
+      <c r="K6" s="71" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" s="74" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="66" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="67" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="36">
-        <v>1</v>
-      </c>
-      <c r="H7" s="34">
-        <v>0</v>
-      </c>
-      <c r="I7" s="72" t="s">
-        <v>37</v>
-      </c>
-      <c r="J7" s="34">
-        <v>0</v>
-      </c>
-      <c r="K7" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="L7" s="50" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" s="70" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="71" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="34" t="s">
+      <c r="F7" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="37">
+        <v>1</v>
+      </c>
+      <c r="H7" s="35">
+        <v>0</v>
+      </c>
+      <c r="I7" s="68" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="34" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="36" t="s">
+      <c r="J7" s="35">
+        <v>0</v>
+      </c>
+      <c r="K7" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="66" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="67" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="36">
-        <v>1</v>
-      </c>
-      <c r="H8" s="34">
-        <v>0</v>
-      </c>
-      <c r="I8" s="72" t="s">
-        <v>41</v>
-      </c>
-      <c r="J8" s="34">
-        <v>0</v>
-      </c>
-      <c r="K8" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="L8" s="50" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="79"/>
-      <c r="B9" s="34"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="72"/>
-      <c r="J9" s="34"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="50"/>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="A10" s="79"/>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="72"/>
-      <c r="I10" s="72"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="72"/>
-      <c r="L10" s="80"/>
-    </row>
-    <row r="11" ht="14.75" spans="1:12">
-      <c r="A11" s="81"/>
-      <c r="B11" s="82"/>
-      <c r="C11" s="82"/>
-      <c r="D11" s="82"/>
-      <c r="E11" s="82"/>
-      <c r="F11" s="82"/>
-      <c r="G11" s="82"/>
-      <c r="H11" s="83"/>
-      <c r="I11" s="83"/>
-      <c r="J11" s="82"/>
-      <c r="K11" s="83"/>
-      <c r="L11" s="84"/>
+      <c r="F8" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="37">
+        <v>1</v>
+      </c>
+      <c r="H8" s="35">
+        <v>0</v>
+      </c>
+      <c r="I8" s="68" t="s">
+        <v>44</v>
+      </c>
+      <c r="J8" s="35">
+        <v>0</v>
+      </c>
+      <c r="K8" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M8" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="75"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="68"/>
+      <c r="J9" s="35"/>
+      <c r="K9" s="35"/>
+      <c r="L9" s="10"/>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="75"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="68"/>
+      <c r="I10" s="68"/>
+      <c r="J10" s="35"/>
+      <c r="K10" s="68"/>
+      <c r="L10" s="76"/>
+    </row>
+    <row r="11" ht="14.75" spans="1:13">
+      <c r="A11" s="77"/>
+      <c r="B11" s="78"/>
+      <c r="C11" s="78"/>
+      <c r="D11" s="78"/>
+      <c r="E11" s="78"/>
+      <c r="F11" s="78"/>
+      <c r="G11" s="78"/>
+      <c r="H11" s="79"/>
+      <c r="I11" s="79"/>
+      <c r="J11" s="78"/>
+      <c r="K11" s="79"/>
+      <c r="L11" s="80"/>
     </row>
     <row r="12" ht="14.75"/>
   </sheetData>
+  <conditionalFormatting sqref="M2:M8">
+    <cfRule type="expression" dxfId="12" priority="1">
+      <formula>$M2="False"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
@@ -4344,347 +4317,347 @@
   <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.90909090909091" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="26.5454545454545" style="29" customWidth="1"/>
-    <col min="2" max="2" width="26.8181818181818" style="29" customWidth="1"/>
-    <col min="3" max="3" width="15.8181818181818" style="29" customWidth="1"/>
-    <col min="4" max="4" width="96.8181818181818" style="29" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="18.1818181818182" style="29" customWidth="1"/>
-    <col min="6" max="6" width="19.0909090909091" style="29" customWidth="1"/>
-    <col min="7" max="7" width="9" style="29" customWidth="1"/>
-    <col min="8" max="8" width="8.90909090909091" style="29"/>
-    <col min="9" max="9" width="9.54545454545454" style="29" customWidth="1"/>
-    <col min="10" max="12" width="8.90909090909091" style="29"/>
-    <col min="13" max="13" width="15.1818181818182" style="29" customWidth="1"/>
-    <col min="14" max="14" width="19.7636363636364" style="29" customWidth="1"/>
-    <col min="15" max="16384" width="8.90909090909091" style="29"/>
+    <col min="1" max="1" width="26.5454545454545" style="30" customWidth="1"/>
+    <col min="2" max="2" width="26.8181818181818" style="30" customWidth="1"/>
+    <col min="3" max="3" width="15.8181818181818" style="30" customWidth="1"/>
+    <col min="4" max="4" width="96.8181818181818" style="30" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="18.1818181818182" style="30" customWidth="1"/>
+    <col min="6" max="6" width="19.0909090909091" style="30" customWidth="1"/>
+    <col min="7" max="7" width="9" style="30" customWidth="1"/>
+    <col min="8" max="8" width="8.90909090909091" style="30"/>
+    <col min="9" max="9" width="9.54545454545454" style="30" customWidth="1"/>
+    <col min="10" max="12" width="8.90909090909091" style="30"/>
+    <col min="13" max="13" width="15.1818181818182" style="30" customWidth="1"/>
+    <col min="14" max="14" width="19.7636363636364" style="30" customWidth="1"/>
+    <col min="15" max="16384" width="8.90909090909091" style="30"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="14.75" spans="1:14">
-      <c r="A1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="44" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="44" t="s">
+      <c r="A1" s="44" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="45" t="s">
+      <c r="D1" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="44" t="s">
+      <c r="F1" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="44" t="s">
+      <c r="G1" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="46" t="s">
+      <c r="H1" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="44" t="s">
-        <v>42</v>
-      </c>
-      <c r="J1" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="K1" s="44" t="s">
+      <c r="I1" s="45" t="s">
+        <v>45</v>
+      </c>
+      <c r="J1" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="K1" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="44" t="s">
+      <c r="L1" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="48" t="s">
+      <c r="M1" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="48" t="s">
+      <c r="N1" s="49" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="35" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" s="37">
+        <v>1</v>
+      </c>
+      <c r="H2" s="35">
+        <v>0</v>
+      </c>
+      <c r="I2" s="35">
+        <v>2</v>
+      </c>
+      <c r="J2" s="35">
+        <v>1</v>
+      </c>
+      <c r="K2" s="35">
+        <v>0</v>
+      </c>
+      <c r="L2" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M2" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" s="37">
+        <v>1</v>
+      </c>
+      <c r="H3" s="35">
+        <v>0</v>
+      </c>
+      <c r="I3" s="35">
+        <v>3</v>
+      </c>
+      <c r="J3" s="35">
+        <v>1</v>
+      </c>
+      <c r="K3" s="35">
+        <v>0</v>
+      </c>
+      <c r="L3" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M3" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N3" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="50" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="35" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2" s="49" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" s="34" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="37" t="s">
-        <v>47</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G2" s="36">
-        <v>1</v>
-      </c>
-      <c r="H2" s="34">
-        <v>0</v>
-      </c>
-      <c r="I2" s="34">
+      <c r="F4" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="G4" s="37">
+        <v>1</v>
+      </c>
+      <c r="H4" s="35">
+        <v>0</v>
+      </c>
+      <c r="I4" s="35">
         <v>2</v>
       </c>
-      <c r="J2" s="34">
-        <v>1</v>
-      </c>
-      <c r="K2" s="34">
-        <v>0</v>
-      </c>
-      <c r="L2" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M2" s="50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N2" s="50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3" s="49" t="s">
+      <c r="J4" s="35">
+        <v>2</v>
+      </c>
+      <c r="K4" s="35">
+        <v>0</v>
+      </c>
+      <c r="L4" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N4" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="50" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="G5" s="37">
+        <v>1</v>
+      </c>
+      <c r="H5" s="35">
+        <v>0</v>
+      </c>
+      <c r="I5" s="35">
+        <v>3</v>
+      </c>
+      <c r="J5" s="35">
+        <v>2</v>
+      </c>
+      <c r="K5" s="35">
+        <v>0</v>
+      </c>
+      <c r="L5" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="50" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="34" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" s="37" t="s">
-        <v>52</v>
-      </c>
-      <c r="E3" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G3" s="36">
-        <v>1</v>
-      </c>
-      <c r="H3" s="34">
-        <v>0</v>
-      </c>
-      <c r="I3" s="34">
-        <v>3</v>
-      </c>
-      <c r="J3" s="34">
-        <v>1</v>
-      </c>
-      <c r="K3" s="34">
-        <v>0</v>
-      </c>
-      <c r="L3" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M3" s="50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N3" s="50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4" s="49" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" s="37" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G4" s="36">
-        <v>1</v>
-      </c>
-      <c r="H4" s="34">
-        <v>0</v>
-      </c>
-      <c r="I4" s="34">
+      <c r="G6" s="37">
+        <v>1</v>
+      </c>
+      <c r="H6" s="35">
+        <v>0</v>
+      </c>
+      <c r="I6" s="35">
+        <v>5</v>
+      </c>
+      <c r="J6" s="35">
+        <v>1</v>
+      </c>
+      <c r="K6" s="35">
+        <v>0</v>
+      </c>
+      <c r="L6" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="50" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="37">
+        <v>1</v>
+      </c>
+      <c r="H7" s="35">
+        <v>0</v>
+      </c>
+      <c r="I7" s="35">
+        <v>5</v>
+      </c>
+      <c r="J7" s="35">
         <v>2</v>
       </c>
-      <c r="J4" s="34">
-        <v>2</v>
-      </c>
-      <c r="K4" s="34">
-        <v>0</v>
-      </c>
-      <c r="L4" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M4" s="50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N4" s="50" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="A5" s="49" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="37" t="s">
-        <v>52</v>
-      </c>
-      <c r="E5" s="34" t="s">
-        <v>58</v>
-      </c>
-      <c r="F5" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G5" s="36">
-        <v>1</v>
-      </c>
-      <c r="H5" s="34">
-        <v>0</v>
-      </c>
-      <c r="I5" s="34">
-        <v>3</v>
-      </c>
-      <c r="J5" s="34">
-        <v>2</v>
-      </c>
-      <c r="K5" s="34">
-        <v>0</v>
-      </c>
-      <c r="L5" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M5" s="50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N5" s="50" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
-      <c r="A6" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="C6" s="34" t="s">
-        <v>60</v>
-      </c>
-      <c r="D6" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="E6" s="34" t="s">
-        <v>62</v>
-      </c>
-      <c r="F6" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G6" s="36">
-        <v>1</v>
-      </c>
-      <c r="H6" s="34">
-        <v>0</v>
-      </c>
-      <c r="I6" s="34">
-        <v>5</v>
-      </c>
-      <c r="J6" s="34">
-        <v>1</v>
-      </c>
-      <c r="K6" s="34">
-        <v>0</v>
-      </c>
-      <c r="L6" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M6" s="50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N6" s="50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="D7" s="37" t="s">
-        <v>61</v>
-      </c>
-      <c r="E7" s="34" t="s">
-        <v>65</v>
-      </c>
-      <c r="F7" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" s="36">
-        <v>1</v>
-      </c>
-      <c r="H7" s="34">
-        <v>0</v>
-      </c>
-      <c r="I7" s="34">
-        <v>5</v>
-      </c>
-      <c r="J7" s="34">
-        <v>2</v>
-      </c>
-      <c r="K7" s="34">
-        <v>0</v>
-      </c>
-      <c r="L7" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M7" s="50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N7" s="50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" s="41" customFormat="1" spans="1:14">
+      <c r="K7" s="35">
+        <v>0</v>
+      </c>
+      <c r="L7" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" s="42" customFormat="1" spans="1:14">
       <c r="A8" s="51" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C8" s="53" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D8" s="54" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E8" s="55" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F8" s="53" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G8" s="53">
         <v>1</v>
@@ -4707,52 +4680,52 @@
       <c r="M8" s="56" t="b">
         <v>0</v>
       </c>
-      <c r="N8" s="50" t="s">
-        <v>55</v>
+      <c r="N8" s="10" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:14">
-      <c r="A9" s="49" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="C9" s="34" t="s">
+      <c r="A9" s="50" t="s">
         <v>72</v>
       </c>
-      <c r="D9" s="37" t="s">
+      <c r="B9" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="35" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="36">
-        <v>1</v>
-      </c>
-      <c r="H9" s="34">
-        <v>0</v>
-      </c>
-      <c r="I9" s="34">
+      <c r="D9" s="38" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="37">
+        <v>1</v>
+      </c>
+      <c r="H9" s="35">
+        <v>0</v>
+      </c>
+      <c r="I9" s="35">
         <v>4</v>
       </c>
-      <c r="J9" s="34">
-        <v>1</v>
-      </c>
-      <c r="K9" s="34">
-        <v>0</v>
-      </c>
-      <c r="L9" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M9" s="50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N9" s="50" t="s">
-        <v>74</v>
+      <c r="J9" s="35">
+        <v>1</v>
+      </c>
+      <c r="K9" s="35">
+        <v>0</v>
+      </c>
+      <c r="L9" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N9" s="10" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -4769,10 +4742,10 @@
         <v>77</v>
       </c>
       <c r="E10" s="61" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F10" s="59" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G10" s="59">
         <v>1</v>
@@ -4795,51 +4768,51 @@
       <c r="M10" s="62" t="b">
         <v>1</v>
       </c>
-      <c r="N10" s="50" t="s">
+      <c r="N10" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" s="38" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="11" spans="1:14">
-      <c r="A11" s="49" t="s">
-        <v>78</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="D11" s="37" t="s">
-        <v>73</v>
-      </c>
-      <c r="E11" s="34" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G11" s="36">
-        <v>1</v>
-      </c>
-      <c r="H11" s="34">
-        <v>0</v>
-      </c>
-      <c r="I11" s="34">
+      <c r="E11" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11" s="37">
+        <v>1</v>
+      </c>
+      <c r="H11" s="35">
+        <v>0</v>
+      </c>
+      <c r="I11" s="35">
         <v>4</v>
       </c>
-      <c r="J11" s="34">
+      <c r="J11" s="35">
         <v>2</v>
       </c>
-      <c r="K11" s="34">
-        <v>0</v>
-      </c>
-      <c r="L11" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M11" s="50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N11" s="50" t="s">
+      <c r="K11" s="35">
+        <v>0</v>
+      </c>
+      <c r="L11" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N11" s="10" t="s">
         <v>80</v>
       </c>
     </row>
@@ -4857,10 +4830,10 @@
         <v>83</v>
       </c>
       <c r="E12" s="61" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F12" s="59" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G12" s="59">
         <v>1</v>
@@ -4881,52 +4854,52 @@
       <c r="M12" s="62" t="b">
         <v>1</v>
       </c>
-      <c r="N12" s="50" t="s">
+      <c r="N12" s="10" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:14">
-      <c r="A13" s="49" t="s">
+      <c r="A13" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C13" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="D13" s="37" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G13" s="36">
-        <v>1</v>
-      </c>
-      <c r="H13" s="34">
-        <v>0</v>
-      </c>
-      <c r="I13" s="34">
+      <c r="D13" s="38" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="G13" s="37">
+        <v>1</v>
+      </c>
+      <c r="H13" s="35">
+        <v>0</v>
+      </c>
+      <c r="I13" s="35">
         <v>6</v>
       </c>
-      <c r="J13" s="34">
+      <c r="J13" s="35">
         <v>2</v>
       </c>
-      <c r="K13" s="34">
-        <v>0</v>
-      </c>
-      <c r="L13" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M13" s="50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N13" s="50" t="s">
-        <v>74</v>
+      <c r="K13" s="35">
+        <v>0</v>
+      </c>
+      <c r="L13" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M13" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N13" s="10" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -4946,7 +4919,7 @@
         <v>88</v>
       </c>
       <c r="F14" s="59" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G14" s="59">
         <v>1</v>
@@ -4969,55 +4942,55 @@
       <c r="M14" s="62" t="b">
         <v>1</v>
       </c>
-      <c r="N14" s="50" t="s">
-        <v>74</v>
+      <c r="N14" s="10" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:14">
-      <c r="A15" s="49" t="s">
+      <c r="A15" s="50" t="s">
         <v>89</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="C15" s="34" t="s">
+      <c r="C15" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="D15" s="37" t="s">
-        <v>69</v>
-      </c>
-      <c r="E15" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="F15" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G15" s="36">
-        <v>1</v>
-      </c>
-      <c r="H15" s="34">
-        <v>0</v>
-      </c>
-      <c r="I15" s="34">
+      <c r="D15" s="38" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="F15" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="37">
+        <v>1</v>
+      </c>
+      <c r="H15" s="35">
+        <v>0</v>
+      </c>
+      <c r="I15" s="35">
         <v>7</v>
       </c>
-      <c r="J15" s="34">
+      <c r="J15" s="35">
         <v>3</v>
       </c>
-      <c r="K15" s="34">
-        <v>0</v>
-      </c>
-      <c r="L15" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M15" s="50" t="b">
-        <v>1</v>
-      </c>
-      <c r="N15" s="50" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" s="41" customFormat="1" spans="1:14">
+      <c r="K15" s="35">
+        <v>0</v>
+      </c>
+      <c r="L15" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M15" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" s="42" customFormat="1" spans="1:14">
       <c r="A16" s="51" t="s">
         <v>91</v>
       </c>
@@ -5028,13 +5001,13 @@
         <v>92</v>
       </c>
       <c r="D16" s="54" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E16" s="55" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F16" s="55" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G16" s="55">
         <v>1</v>
@@ -5057,9 +5030,11 @@
       <c r="M16" s="56" t="b">
         <v>0</v>
       </c>
-      <c r="N16" s="56"/>
-    </row>
-    <row r="17" s="42" customFormat="1" ht="28" spans="1:14">
+      <c r="N16" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" s="43" customFormat="1" ht="28" spans="1:14">
       <c r="A17" s="51" t="s">
         <v>93</v>
       </c>
@@ -5076,7 +5051,7 @@
         <v>96</v>
       </c>
       <c r="F17" s="52" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G17" s="52">
         <v>3</v>
@@ -5099,64 +5074,68 @@
       <c r="M17" s="64" t="b">
         <v>0</v>
       </c>
-      <c r="N17" s="64"/>
-    </row>
-    <row r="18" s="41" customFormat="1" ht="31.25" customHeight="1" spans="1:14">
-      <c r="A18" s="65" t="s">
+      <c r="N17" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" s="42" customFormat="1" ht="31.25" customHeight="1" spans="1:14">
+      <c r="A18" s="51" t="s">
         <v>97</v>
       </c>
-      <c r="B18" s="66" t="s">
+      <c r="B18" s="52" t="s">
         <v>97</v>
       </c>
-      <c r="C18" s="66" t="s">
+      <c r="C18" s="52" t="s">
         <v>98</v>
       </c>
-      <c r="D18" s="67" t="s">
+      <c r="D18" s="63" t="s">
         <v>99</v>
       </c>
-      <c r="E18" s="68" t="s">
-        <v>21</v>
-      </c>
-      <c r="F18" s="66" t="s">
-        <v>48</v>
-      </c>
-      <c r="G18" s="66">
-        <v>1</v>
-      </c>
-      <c r="H18" s="68">
-        <v>0</v>
-      </c>
-      <c r="I18" s="68">
+      <c r="E18" s="55" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="52" t="s">
+        <v>50</v>
+      </c>
+      <c r="G18" s="65">
+        <v>1</v>
+      </c>
+      <c r="H18" s="55">
+        <v>0</v>
+      </c>
+      <c r="I18" s="55">
         <v>6</v>
       </c>
-      <c r="J18" s="68">
+      <c r="J18" s="55">
         <v>2</v>
       </c>
-      <c r="K18" s="68">
-        <v>0</v>
-      </c>
-      <c r="L18" s="66" t="b">
-        <v>0</v>
-      </c>
-      <c r="M18" s="69" t="b">
-        <v>0</v>
-      </c>
-      <c r="N18" s="69"/>
+      <c r="K18" s="55">
+        <v>0</v>
+      </c>
+      <c r="L18" s="52" t="b">
+        <v>0</v>
+      </c>
+      <c r="M18" s="64" t="b">
+        <v>0</v>
+      </c>
+      <c r="N18" s="10" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="19" ht="14.75"/>
   </sheetData>
   <conditionalFormatting sqref="F17:F18">
-    <cfRule type="expression" dxfId="24" priority="3">
+    <cfRule type="expression" dxfId="25" priority="3">
       <formula>$F17="Self"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F18 F19:G59">
-    <cfRule type="expression" dxfId="25" priority="2">
+    <cfRule type="expression" dxfId="26" priority="2">
       <formula>$F2="Enemy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M78 N2:N18">
-    <cfRule type="expression" dxfId="26" priority="1">
+    <cfRule type="expression" dxfId="12" priority="1">
       <formula>$M2="False"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5172,197 +5151,217 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultColWidth="8.90909090909091" defaultRowHeight="14" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="20" style="29" customWidth="1"/>
-    <col min="2" max="2" width="17.8181818181818" style="29" customWidth="1"/>
-    <col min="3" max="3" width="8.90909090909091" style="29"/>
-    <col min="4" max="4" width="48.4545454545455" style="29" customWidth="1"/>
-    <col min="5" max="5" width="8.90909090909091" style="29"/>
-    <col min="6" max="7" width="17.3636363636364" style="29" customWidth="1"/>
-    <col min="8" max="8" width="8.90909090909091" style="29"/>
-    <col min="9" max="9" width="12.0909090909091" style="29" customWidth="1"/>
-    <col min="10" max="10" width="13.4545454545455" style="29" customWidth="1"/>
-    <col min="11" max="16384" width="8.90909090909091" style="29"/>
+    <col min="1" max="1" width="20" style="30" customWidth="1"/>
+    <col min="2" max="2" width="17.8181818181818" style="30" customWidth="1"/>
+    <col min="3" max="3" width="8.90909090909091" style="30"/>
+    <col min="4" max="4" width="48.4545454545455" style="30" customWidth="1"/>
+    <col min="5" max="5" width="8.90909090909091" style="30"/>
+    <col min="6" max="7" width="17.3636363636364" style="30" customWidth="1"/>
+    <col min="8" max="8" width="8.90909090909091" style="30"/>
+    <col min="9" max="9" width="12.0909090909091" style="30" customWidth="1"/>
+    <col min="10" max="10" width="13.4545454545455" style="30" customWidth="1"/>
+    <col min="11" max="16384" width="8.90909090909091" style="30"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="30" t="s">
+    <row r="1" spans="1:12">
+      <c r="A1" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="30" t="s">
+      <c r="E1" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="30" t="s">
+      <c r="F1" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="30" t="s">
+      <c r="G1" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="33" t="s">
+      <c r="I1" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="33" t="s">
+      <c r="J1" s="34" t="s">
         <v>10</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="14" t="s">
+      <c r="L1" s="30" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="C2" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="D2" s="37" t="s">
+      <c r="D2" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="34" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="36" t="s">
+      <c r="E2" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="36">
-        <v>1</v>
-      </c>
-      <c r="H2" s="34">
-        <v>0</v>
-      </c>
-      <c r="I2" s="34">
-        <v>0</v>
-      </c>
-      <c r="J2" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="K2" s="34" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="14" t="s">
+      <c r="F2" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="37">
+        <v>1</v>
+      </c>
+      <c r="H2" s="35">
+        <v>0</v>
+      </c>
+      <c r="I2" s="35">
+        <v>0</v>
+      </c>
+      <c r="J2" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="K2" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="14" t="s">
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="37">
+        <v>1</v>
+      </c>
+      <c r="H3" s="35">
+        <v>0</v>
+      </c>
+      <c r="I3" s="35">
+        <v>0</v>
+      </c>
+      <c r="J3" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="K3" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="D3" s="37" t="s">
-        <v>105</v>
-      </c>
-      <c r="E3" s="34" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="36" t="s">
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>108</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="E4" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="36">
-        <v>1</v>
-      </c>
-      <c r="H3" s="34">
-        <v>0</v>
-      </c>
-      <c r="I3" s="34">
-        <v>0</v>
-      </c>
-      <c r="J3" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="K3" s="34" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="D4" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="E4" s="34" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="36" t="s">
+      <c r="F4" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="37">
+        <v>1</v>
+      </c>
+      <c r="H4" s="35">
+        <v>0</v>
+      </c>
+      <c r="I4" s="35">
+        <v>0</v>
+      </c>
+      <c r="J4" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="K4" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" s="30" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="39" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="E5" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="36">
-        <v>1</v>
-      </c>
-      <c r="H4" s="34">
-        <v>0</v>
-      </c>
-      <c r="I4" s="34">
-        <v>0</v>
-      </c>
-      <c r="J4" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="K4" s="34" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="24" t="s">
-        <v>109</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>109</v>
-      </c>
-      <c r="C5" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="D5" s="39" t="s">
-        <v>111</v>
-      </c>
-      <c r="E5" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="40">
-        <v>1</v>
-      </c>
-      <c r="H5" s="38">
-        <v>0</v>
-      </c>
-      <c r="I5" s="38">
-        <v>0</v>
-      </c>
-      <c r="J5" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="K5" s="38" t="b">
-        <v>1</v>
+      <c r="F5" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="41">
+        <v>1</v>
+      </c>
+      <c r="H5" s="39">
+        <v>0</v>
+      </c>
+      <c r="I5" s="39">
+        <v>0</v>
+      </c>
+      <c r="J5" s="39" t="b">
+        <v>0</v>
+      </c>
+      <c r="K5" s="39" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" s="30" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="L2:L3">
+    <cfRule type="expression" dxfId="12" priority="1">
+      <formula>$M2="False"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
@@ -5375,195 +5374,215 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultColWidth="8.90909090909091" defaultRowHeight="14" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="28.0909090909091" style="29" customWidth="1"/>
-    <col min="2" max="2" width="29" style="29" customWidth="1"/>
-    <col min="3" max="3" width="8.90909090909091" style="29"/>
-    <col min="4" max="4" width="71.8181818181818" style="29" customWidth="1"/>
-    <col min="5" max="5" width="10.9090909090909" style="29" customWidth="1"/>
-    <col min="6" max="6" width="8.90909090909091" style="29"/>
-    <col min="7" max="7" width="16.0909090909091" style="29" customWidth="1"/>
-    <col min="8" max="16384" width="8.90909090909091" style="29"/>
+    <col min="1" max="1" width="28.0909090909091" style="30" customWidth="1"/>
+    <col min="2" max="2" width="29" style="30" customWidth="1"/>
+    <col min="3" max="3" width="8.90909090909091" style="30"/>
+    <col min="4" max="4" width="71.8181818181818" style="30" customWidth="1"/>
+    <col min="5" max="5" width="10.9090909090909" style="30" customWidth="1"/>
+    <col min="6" max="6" width="8.90909090909091" style="30"/>
+    <col min="7" max="7" width="16.0909090909091" style="30" customWidth="1"/>
+    <col min="8" max="16384" width="8.90909090909091" style="30"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" s="30" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="30" t="s">
+    <row r="1" spans="1:12">
+      <c r="A1" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="30" t="s">
+      <c r="E1" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="30" t="s">
+      <c r="F1" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="30" t="s">
+      <c r="G1" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="33" t="s">
+      <c r="I1" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="33" t="s">
+      <c r="J1" s="34" t="s">
         <v>10</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="C2" s="34" t="s">
+      <c r="L1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="35" t="s">
+      <c r="B2" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="D2" s="36" t="s">
+        <v>115</v>
+      </c>
+      <c r="E2" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="36" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="36">
-        <v>1</v>
-      </c>
-      <c r="H2" s="34">
-        <v>0</v>
-      </c>
-      <c r="I2" s="34">
-        <v>0</v>
-      </c>
-      <c r="J2" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="K2" s="34" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="C3" s="34" t="s">
+      <c r="G2" s="37">
+        <v>1</v>
+      </c>
+      <c r="H2" s="35">
+        <v>0</v>
+      </c>
+      <c r="I2" s="35">
+        <v>0</v>
+      </c>
+      <c r="J2" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="K2" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="B3" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" s="35" t="s">
         <v>117</v>
       </c>
-      <c r="E3" s="34" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="36" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="36">
-        <v>1</v>
-      </c>
-      <c r="H3" s="34">
-        <v>0</v>
-      </c>
-      <c r="I3" s="34">
-        <v>0</v>
-      </c>
-      <c r="J3" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="K3" s="34" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="14" t="s">
+      <c r="D3" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="C4" s="34" t="s">
+      <c r="E3" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="37">
+        <v>1</v>
+      </c>
+      <c r="H3" s="35">
+        <v>0</v>
+      </c>
+      <c r="I3" s="35">
+        <v>0</v>
+      </c>
+      <c r="J3" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="K3" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="B4" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="C4" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="D4" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="F4" s="36" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="36">
-        <v>1</v>
-      </c>
-      <c r="H4" s="34">
-        <v>0</v>
-      </c>
-      <c r="I4" s="34">
-        <v>0</v>
-      </c>
-      <c r="J4" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="K4" s="34" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="24" t="s">
+      <c r="E4" s="35" t="s">
         <v>122</v>
       </c>
-      <c r="B5" s="24" t="s">
-        <v>122</v>
-      </c>
-      <c r="C5" s="38" t="s">
+      <c r="F4" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="37">
+        <v>1</v>
+      </c>
+      <c r="H4" s="35">
+        <v>0</v>
+      </c>
+      <c r="I4" s="35">
+        <v>0</v>
+      </c>
+      <c r="J4" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="K4" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" s="30" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="B5" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="C5" s="39" t="s">
         <v>124</v>
       </c>
-      <c r="E5" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="F5" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="40">
-        <v>1</v>
-      </c>
-      <c r="H5" s="38">
-        <v>0</v>
-      </c>
-      <c r="I5" s="38">
-        <v>0</v>
-      </c>
-      <c r="J5" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="K5" s="38" t="b">
-        <v>1</v>
+      <c r="D5" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" s="39" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="41">
+        <v>1</v>
+      </c>
+      <c r="H5" s="39">
+        <v>0</v>
+      </c>
+      <c r="I5" s="39">
+        <v>0</v>
+      </c>
+      <c r="J5" s="39" t="b">
+        <v>0</v>
+      </c>
+      <c r="K5" s="39" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" s="30" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="L2:L3">
+    <cfRule type="expression" dxfId="12" priority="1">
+      <formula>$M2="False"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <tableParts count="1">
@@ -5575,7 +5594,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr defaultColWidth="8.90909090909091" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="2" width="28.0909090909091" style="1" customWidth="1"/>
@@ -5590,7 +5609,7 @@
     <col min="13" max="16384" width="8.90909090909091" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5613,7 +5632,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>7</v>
@@ -5627,650 +5646,664 @@
       <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F2" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="7">
+        <v>1</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="I2" s="7">
+        <v>1</v>
+      </c>
+      <c r="J2" s="7">
+        <v>0</v>
+      </c>
+      <c r="K2" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="7">
-        <v>1</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="I2" s="7">
-        <v>1</v>
-      </c>
-      <c r="J2" s="7">
-        <v>0</v>
-      </c>
-      <c r="K2" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="L2" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" s="7" t="s">
+      <c r="F3" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" s="7">
+        <v>1</v>
+      </c>
+      <c r="H3" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="I3" s="7">
+        <v>1</v>
+      </c>
+      <c r="J3" s="7">
+        <v>0</v>
+      </c>
+      <c r="K3" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="15">
+        <v>0</v>
+      </c>
+      <c r="H4" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G3" s="7">
-        <v>1</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="I3" s="7">
-        <v>1</v>
-      </c>
-      <c r="J3" s="7">
-        <v>0</v>
-      </c>
-      <c r="K3" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="L3" s="7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="A4" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" s="14" t="s">
+      <c r="I4" s="15">
+        <v>0</v>
+      </c>
+      <c r="J4" s="15">
+        <v>0</v>
+      </c>
+      <c r="K4" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" s="16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="15">
+        <v>0</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="I5" s="15">
+        <v>4</v>
+      </c>
+      <c r="J5" s="15">
+        <v>0</v>
+      </c>
+      <c r="K5" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>142</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="15">
+        <v>1</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="I6" s="15">
+        <v>2</v>
+      </c>
+      <c r="J6" s="15">
+        <v>0</v>
+      </c>
+      <c r="K6" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="15">
+        <v>1</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="I7" s="15">
+        <v>2</v>
+      </c>
+      <c r="J7" s="15">
+        <v>0</v>
+      </c>
+      <c r="K7" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" ht="28" spans="1:13">
+      <c r="A8" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="15">
+        <v>0</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="I8" s="15">
+        <v>3</v>
+      </c>
+      <c r="J8" s="15">
+        <v>0</v>
+      </c>
+      <c r="K8" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="E9" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="14">
-        <v>0</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I4" s="14">
-        <v>0</v>
-      </c>
-      <c r="J4" s="14">
-        <v>0</v>
-      </c>
-      <c r="K4" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L4" s="15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="16" t="s">
-        <v>136</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>136</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="F5" s="14" t="s">
+      <c r="F9" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="15">
+        <v>0</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="I9" s="15">
+        <v>3</v>
+      </c>
+      <c r="J9" s="15">
+        <v>0</v>
+      </c>
+      <c r="K9" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L9" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="28" spans="1:13">
+      <c r="A10" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="G10" s="15">
+        <v>1</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="I10" s="15">
+        <v>0</v>
+      </c>
+      <c r="J10" s="15">
+        <v>0</v>
+      </c>
+      <c r="K10" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" ht="28" spans="1:13">
+      <c r="A11" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="G11" s="15">
+        <v>2</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="I11" s="15">
+        <v>0</v>
+      </c>
+      <c r="J11" s="15">
+        <v>0</v>
+      </c>
+      <c r="K11" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L11" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
+      <c r="A12" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="15">
+        <v>0</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="I12" s="15">
+        <v>8</v>
+      </c>
+      <c r="J12" s="15">
+        <v>0</v>
+      </c>
+      <c r="K12" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L12" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="G13" s="15">
+        <v>1</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="I13" s="15">
+        <v>5</v>
+      </c>
+      <c r="J13" s="15">
+        <v>0</v>
+      </c>
+      <c r="K13" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L13" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="52" spans="1:13">
+      <c r="A14" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="E14" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="14">
-        <v>0</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I5" s="14">
-        <v>4</v>
-      </c>
-      <c r="J5" s="14">
-        <v>0</v>
-      </c>
-      <c r="K5" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L5" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>142</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="G6" s="14">
-        <v>1</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I6" s="14">
-        <v>2</v>
-      </c>
-      <c r="J6" s="14">
-        <v>0</v>
-      </c>
-      <c r="K6" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L6" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" s="14">
-        <v>1</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I7" s="14">
-        <v>2</v>
-      </c>
-      <c r="J7" s="14">
-        <v>0</v>
-      </c>
-      <c r="K7" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L7" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" ht="28" spans="1:12">
-      <c r="A8" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>148</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" s="14">
-        <v>0</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I8" s="14">
+      <c r="F14" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="15">
+        <v>0</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="I14" s="15">
+        <v>0</v>
+      </c>
+      <c r="J14" s="15">
+        <v>0</v>
+      </c>
+      <c r="K14" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L14" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>173</v>
+      </c>
+      <c r="D15" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>175</v>
+      </c>
+      <c r="F15" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" s="15">
+        <v>0</v>
+      </c>
+      <c r="H15" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="I15" s="25">
         <v>3</v>
       </c>
-      <c r="J8" s="14">
-        <v>0</v>
-      </c>
-      <c r="K8" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L8" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="14">
-        <v>0</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I9" s="14">
-        <v>3</v>
-      </c>
-      <c r="J9" s="14">
-        <v>0</v>
-      </c>
-      <c r="K9" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L9" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" ht="28" spans="1:12">
-      <c r="A10" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>154</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>155</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="G10" s="14">
-        <v>1</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I10" s="14">
-        <v>0</v>
-      </c>
-      <c r="J10" s="14">
-        <v>0</v>
-      </c>
-      <c r="K10" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L10" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" ht="28" spans="1:12">
-      <c r="A11" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>159</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="G11" s="14">
-        <v>2</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I11" s="14">
-        <v>0</v>
-      </c>
-      <c r="J11" s="14">
-        <v>0</v>
-      </c>
-      <c r="K11" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L11" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="F12" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G12" s="14">
-        <v>0</v>
-      </c>
-      <c r="H12" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I12" s="14">
-        <v>8</v>
-      </c>
-      <c r="J12" s="14">
-        <v>0</v>
-      </c>
-      <c r="K12" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L12" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="A13" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>167</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="G13" s="14">
-        <v>1</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I13" s="14">
-        <v>5</v>
-      </c>
-      <c r="J13" s="14">
-        <v>0</v>
-      </c>
-      <c r="K13" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L13" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" ht="52" spans="1:12">
-      <c r="A14" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" s="14">
-        <v>0</v>
-      </c>
-      <c r="H14" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I14" s="14">
-        <v>0</v>
-      </c>
-      <c r="J14" s="14">
-        <v>0</v>
-      </c>
-      <c r="K14" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L14" s="14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
-      <c r="A15" s="24" t="s">
-        <v>171</v>
-      </c>
-      <c r="B15" s="24" t="s">
-        <v>171</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>172</v>
-      </c>
-      <c r="D15" s="25" t="s">
-        <v>173</v>
-      </c>
-      <c r="E15" s="24" t="s">
-        <v>174</v>
-      </c>
-      <c r="F15" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="G15" s="14">
-        <v>0</v>
-      </c>
-      <c r="H15" s="24" t="s">
-        <v>129</v>
-      </c>
-      <c r="I15" s="24">
-        <v>3</v>
-      </c>
-      <c r="J15" s="24">
-        <v>0</v>
-      </c>
-      <c r="K15" s="24" t="b">
-        <v>0</v>
-      </c>
-      <c r="L15" s="24" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12">
-      <c r="A16" s="26"/>
-      <c r="B16" s="26"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="28"/>
+      <c r="J15" s="25">
+        <v>0</v>
+      </c>
+      <c r="K15" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" s="25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="A16" s="27"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="29"/>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" s="26"/>
-      <c r="B17" s="26"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="28"/>
+      <c r="A17" s="27"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="29"/>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" s="26"/>
-      <c r="B18" s="26"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="28"/>
+      <c r="A18" s="27"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="29"/>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="26"/>
-      <c r="B19" s="26"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="28"/>
+      <c r="A19" s="27"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="29"/>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" s="26"/>
-      <c r="B20" s="26"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="28"/>
+      <c r="A20" s="27"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="29"/>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="26"/>
-      <c r="B21" s="26"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="28"/>
+      <c r="A21" s="27"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="29"/>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="26"/>
-      <c r="B22" s="26"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="28"/>
+      <c r="A22" s="27"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="29"/>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" s="26"/>
-      <c r="B23" s="26"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="28"/>
+      <c r="A23" s="27"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="29"/>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="26"/>
-      <c r="B24" s="26"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="28"/>
+      <c r="A24" s="27"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="29"/>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="26"/>
-      <c r="B25" s="26"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="28"/>
+      <c r="A25" s="27"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="29"/>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" s="26"/>
-      <c r="B26" s="26"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="28"/>
+      <c r="A26" s="27"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="29"/>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" s="26"/>
-      <c r="B27" s="26"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="28"/>
+      <c r="A27" s="27"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="29"/>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" s="26"/>
-      <c r="B28" s="26"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="28"/>
+      <c r="A28" s="27"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="29"/>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="26"/>
-      <c r="B29" s="26"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="28"/>
+      <c r="A29" s="27"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="29"/>
     </row>
     <row r="30" spans="1:4">
-      <c r="A30" s="26"/>
-      <c r="B30" s="26"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="28"/>
+      <c r="A30" s="27"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="29"/>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" s="26"/>
-      <c r="B31" s="26"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="28"/>
+      <c r="A31" s="27"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="29"/>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" s="26"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="28"/>
+      <c r="A32" s="27"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="29"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F15">
-    <cfRule type="expression" dxfId="61" priority="1">
+    <cfRule type="expression" dxfId="61" priority="2">
       <formula>$F2="Null"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F36">
-    <cfRule type="expression" dxfId="24" priority="2">
+    <cfRule type="expression" dxfId="25" priority="3">
       <formula>$F2="Self"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M2:M3">
+    <cfRule type="expression" dxfId="12" priority="1">
+      <formula>$M2="False"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>